<commit_message>
Sorting Sahayak: TD/Non-TD modes, new colours, scan crash fix
- Replace Ordinary/Parcel categories with TD and Non-TD built-in modes;
  hint when a PIN is only in the other mode.
- New navy/teal/amber theme, cleaner keypad and cards.
- Compact "no scheme" bar with Import/Sample; show the post office as the
  main answer when no scheme is active.
- Fix airport codes wrapping at large font sizes.
- Keep ML Kit component registrars from R8 so scanning works in release.
- Sample scheme rebuilt with TD/Non-TD rows; import accepts Line/Route
  columns and office names in the PIN column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J7NCzQ6vFe1yu161DyXRnu
</commit_message>
<xml_diff>
--- a/sorting_sahayak/assets/samples/sample_scheme.xlsx
+++ b/sorting_sahayak/assets/samples/sample_scheme.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="130">
   <si>
     <t xml:space="preserve">SAMPLE – not real. Demo sorting scheme for practice only – replace with your office scheme.</t>
   </si>
@@ -70,313 +70,316 @@
     <t xml:space="preserve">Bag 12</t>
   </si>
   <si>
-    <t xml:space="preserve">Puttur SO</t>
+    <t xml:space="preserve">Puttur Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#D32F2F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sullia Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#2E7D32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574241</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subramanya Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1565C0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">575001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mangaluru HO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#6A1B9A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Udupi HO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#EF6C00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manipal Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#00796B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karkala Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#6D4C41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574299</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puttur group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charmadi Line</t>
   </si>
   <si>
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">#D32F2F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574239</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sullia SO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#2E7D32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574241</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uppinangady SO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#1565C0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">575001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mangaluru HO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#6A1B9A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">576101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Udupi HO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#EF6C00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">576104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manipal SO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#00796B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karkala SO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#6D4C41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">560001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP-BLR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speed Post Bengaluru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speed Post</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Air</t>
+    <t xml:space="preserve">#D81B60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">575030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">City delivery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576299</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kundapura Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#455A64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">574</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puttur Division (other)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#880E4F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">575</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mangaluru NSH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#0097A7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">576</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bag 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Udupi Division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puttur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Articles without PIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sullia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manipal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dakshina Kannada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Udupi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NT-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karnataka – other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-TD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#616161</t>
+  </si>
+  <si>
+    <t xml:space="preserve">56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NT-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bengaluru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NT-41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hubballi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NT-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NT-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chennai</t>
   </si>
   <si>
     <t xml:space="preserve">#F9A825</t>
   </si>
   <si>
-    <t xml:space="preserve">Range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574299</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puttur group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bantwal / Belthangady</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#D81B60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">575030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">City delivery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">576125</t>
-  </si>
-  <si>
-    <t xml:space="preserve">576201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">576299</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kundapura SO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#455A64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">574</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puttur Division (other)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#880E4F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">575</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mangaluru NSH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#0097A7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">576</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Udupi Division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karnataka – other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#616161</t>
-  </si>
-  <si>
-    <t xml:space="preserve">56</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bengaluru NSH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bag 50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southern states</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E</t>
-  </si>
-  <si>
     <t xml:space="preserve">671</t>
   </si>
   <si>
-    <t xml:space="preserve">Bag 60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kasaragod (Kerala)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puttur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Articles without PIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sullia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manipal</t>
+    <t xml:space="preserve">NT-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kannur (Kerala)</t>
   </si>
   <si>
     <t xml:space="preserve">Kasaragod</t>
   </si>
   <si>
-    <t xml:space="preserve">Dakshina Kannada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Udupi</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hassan</t>
   </si>
   <si>
-    <t xml:space="preserve">Bag 31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hassan HO</t>
+    <t xml:space="preserve">NT-31</t>
   </si>
   <si>
     <t xml:space="preserve">Kerala</t>
   </si>
   <si>
-    <t xml:space="preserve">Bag 61</t>
+    <t xml:space="preserve">NT-62</t>
   </si>
   <si>
     <t xml:space="preserve">Kerala – other</t>
   </si>
   <si>
-    <t xml:space="preserve">P-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parcel – Puttur Division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parcel (surface)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surface</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#795548</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AP-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Air parcel – Bengaluru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Air Parcel</t>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NT-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delhi</t>
   </si>
   <si>
     <t xml:space="preserve">#FBC02D</t>
   </si>
   <si>
-    <t xml:space="preserve">60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AP-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Air parcel – Chennai</t>
+    <t xml:space="preserve">40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NT-40M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mumbai</t>
   </si>
   <si>
     <t xml:space="preserve">#FFA000</t>
@@ -385,7 +388,7 @@
     <t xml:space="preserve">Default</t>
   </si>
   <si>
-    <t xml:space="preserve">Bag 99</t>
+    <t xml:space="preserve">NT-99</t>
   </si>
   <si>
     <t xml:space="preserve">All other – send to TMO</t>
@@ -773,13 +776,13 @@
         <v>1</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +790,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -814,13 +817,13 @@
         <v>19</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>1</v>
@@ -834,7 +837,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>1</v>
@@ -855,25 +858,25 @@
         <v>1</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
@@ -881,7 +884,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>1</v>
@@ -902,25 +905,25 @@
         <v>1</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
@@ -928,7 +931,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>1</v>
@@ -949,25 +952,25 @@
         <v>1</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
@@ -975,7 +978,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>1</v>
@@ -996,25 +999,25 @@
         <v>1</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9">
@@ -1022,7 +1025,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>1</v>
@@ -1043,25 +1046,25 @@
         <v>1</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="L9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10">
@@ -1069,7 +1072,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>1</v>
@@ -1090,39 +1093,39 @@
         <v>1</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="L10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>1</v>
@@ -1137,39 +1140,39 @@
         <v>1</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>54</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>1</v>
@@ -1184,39 +1187,39 @@
         <v>1</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>1</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>1</v>
@@ -1231,39 +1234,39 @@
         <v>1</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>62</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>1</v>
@@ -1278,19 +1281,19 @@
         <v>1</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>1</v>
@@ -1301,16 +1304,16 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>1</v>
@@ -1325,42 +1328,42 @@
         <v>1</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="L15" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N15" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>1</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>1</v>
@@ -1372,25 +1375,25 @@
         <v>1</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="L16" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N16" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17">
@@ -1407,7 +1410,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>1</v>
@@ -1419,25 +1422,25 @@
         <v>1</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="L17" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N17" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18">
@@ -1454,7 +1457,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>1</v>
@@ -1466,30 +1469,30 @@
         <v>1</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="L18" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N18" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>78</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>1</v>
@@ -1501,10 +1504,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>1</v>
+        <v>82</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>1</v>
@@ -1513,30 +1516,30 @@
         <v>1</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>81</v>
+        <v>19</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>1</v>
@@ -1548,10 +1551,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>1</v>
@@ -1560,30 +1563,30 @@
         <v>1</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="L20" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>86</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>1</v>
@@ -1595,10 +1598,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>87</v>
+        <v>1</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>1</v>
@@ -1607,30 +1610,30 @@
         <v>1</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="L21" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N21" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>1</v>
@@ -1642,42 +1645,42 @@
         <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>1</v>
+        <v>86</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>1</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>93</v>
+        <v>1</v>
       </c>
       <c r="L22" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N22" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>1</v>
@@ -1689,42 +1692,42 @@
         <v>1</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>1</v>
+        <v>87</v>
       </c>
       <c r="H23" s="1" t="s">
         <v>1</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>93</v>
+        <v>1</v>
       </c>
       <c r="L23" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>1</v>
@@ -1736,10 +1739,10 @@
         <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>97</v>
+        <v>1</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>1</v>
@@ -1748,30 +1751,30 @@
         <v>1</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>98</v>
+        <v>1</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>1</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>1</v>
@@ -1783,10 +1786,10 @@
         <v>1</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>1</v>
+        <v>94</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>1</v>
@@ -1795,30 +1798,30 @@
         <v>1</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>24</v>
+        <v>95</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="L25" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>1</v>
@@ -1830,10 +1833,10 @@
         <v>1</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>1</v>
@@ -1842,30 +1845,30 @@
         <v>1</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N26" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>1</v>
@@ -1877,42 +1880,42 @@
         <v>1</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="F27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>96</v>
-      </c>
       <c r="K27" s="1" t="s">
-        <v>1</v>
+        <v>102</v>
       </c>
       <c r="L27" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>1</v>
@@ -1924,42 +1927,42 @@
         <v>1</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>1</v>
+        <v>103</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G28" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="K28" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="L28" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N28" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>1</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>1</v>
@@ -1971,42 +1974,42 @@
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>103</v>
+        <v>1</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>1</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>1</v>
+        <v>102</v>
       </c>
       <c r="L29" s="1" t="s">
         <v>1</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N29" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>1</v>
@@ -2021,19 +2024,19 @@
         <v>1</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>1</v>
+        <v>110</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>104</v>
+        <v>1</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>1</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>1</v>
@@ -2042,18 +2045,18 @@
         <v>1</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N30" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>1</v>
@@ -2071,16 +2074,16 @@
         <v>1</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>1</v>
+        <v>111</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>1</v>
@@ -2089,18 +2092,18 @@
         <v>1</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N31" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>1</v>
@@ -2112,7 +2115,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>71</v>
+        <v>1</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>1</v>
@@ -2121,13 +2124,13 @@
         <v>1</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>1</v>
+        <v>113</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>1</v>
@@ -2136,13 +2139,13 @@
         <v>1</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>113</v>
+        <v>1</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33">
@@ -2159,7 +2162,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>1</v>
@@ -2171,10 +2174,10 @@
         <v>1</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>1</v>
@@ -2183,13 +2186,13 @@
         <v>1</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34">
@@ -2206,7 +2209,7 @@
         <v>1</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>1</v>
@@ -2218,10 +2221,10 @@
         <v>1</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>1</v>
@@ -2230,18 +2233,18 @@
         <v>1</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>1</v>
@@ -2265,25 +2268,25 @@
         <v>1</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>1</v>
+        <v>92</v>
       </c>
       <c r="N35" s="1" t="s">
         <v>1</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>